<commit_message>
update script + fonctions pour améliorer les résultats obtenus avec gesca
</commit_message>
<xml_diff>
--- a/df_fPC1/sum.var_AMR_EHPAD_C3G_R.xlsx
+++ b/df_fPC1/sum.var_AMR_EHPAD_C3G_R.xlsx
@@ -695,7 +695,7 @@
         <v>-0.0519636488636131</v>
       </c>
       <c r="J2" t="n">
-        <v>0.10036063159044</v>
+        <v>0.103147603373179</v>
       </c>
       <c r="K2" t="n">
         <v>0.0335610808107989</v>
@@ -841,7 +841,7 @@
         <v>0.0110822982171971</v>
       </c>
       <c r="J3" t="n">
-        <v>0.0352159793973484</v>
+        <v>0.0332841500048817</v>
       </c>
       <c r="K3" t="n">
         <v>-0.0975259174762126</v>
@@ -987,7 +987,7 @@
         <v>-0.0181058995709713</v>
       </c>
       <c r="J4" t="n">
-        <v>-0.278648268623139</v>
+        <v>-0.288815238863085</v>
       </c>
       <c r="K4" t="n">
         <v>-0.37338220636912</v>
@@ -1133,7 +1133,7 @@
         <v>-0.0943666974336294</v>
       </c>
       <c r="J5" t="n">
-        <v>-0.046366232871423</v>
+        <v>-0.0408288727958792</v>
       </c>
       <c r="K5" t="n">
         <v>-0.130678648965293</v>
@@ -1279,7 +1279,7 @@
         <v>-0.00777819389424965</v>
       </c>
       <c r="J6" t="n">
-        <v>0.183072132285433</v>
+        <v>0.183906858976229</v>
       </c>
       <c r="K6" t="n">
         <v>-0.0140515295826258</v>
@@ -1425,7 +1425,7 @@
         <v>0.0918115939259928</v>
       </c>
       <c r="J7" t="n">
-        <v>0.0601744798308835</v>
+        <v>0.0530386693634788</v>
       </c>
       <c r="K7" t="n">
         <v>-0.188331569638821</v>
@@ -1571,7 +1571,7 @@
         <v>-0.0493917054781802</v>
       </c>
       <c r="J8" t="n">
-        <v>-0.0883645155060498</v>
+        <v>-0.0853534747701536</v>
       </c>
       <c r="K8" t="n">
         <v>0.309219299525867</v>
@@ -1717,7 +1717,7 @@
         <v>0.0855536155303945</v>
       </c>
       <c r="J9" t="n">
-        <v>0.0504734259398501</v>
+        <v>0.0546274119630951</v>
       </c>
       <c r="K9" t="n">
         <v>-0.208271122741779</v>
@@ -1863,7 +1863,7 @@
         <v>0.0705558338791445</v>
       </c>
       <c r="J10" t="n">
-        <v>0.0849547857042242</v>
+        <v>0.0851385988275439</v>
       </c>
       <c r="K10" t="n">
         <v>0.0601430323680632</v>
@@ -2009,7 +2009,7 @@
         <v>0.0296954906944263</v>
       </c>
       <c r="J11" t="n">
-        <v>0.0158617624856274</v>
+        <v>0.0110290195894473</v>
       </c>
       <c r="K11" t="n">
         <v>0.313060253546427</v>
@@ -2155,7 +2155,7 @@
         <v>0.0663592388653425</v>
       </c>
       <c r="J12" t="n">
-        <v>0.12082021118173</v>
+        <v>0.126087432551128</v>
       </c>
       <c r="K12" t="n">
         <v>0.467253145695357</v>
@@ -2301,7 +2301,7 @@
         <v>-0.133451925871853</v>
       </c>
       <c r="J13" t="n">
-        <v>-0.237554391414924</v>
+        <v>-0.235262158219865</v>
       </c>
       <c r="K13" t="n">
         <v>-0.170995817172662</v>

</xml_diff>